<commit_message>
Add target role to example columns metadata
</commit_message>
<xml_diff>
--- a/data/examples/metadata/ta_columns.xlsx
+++ b/data/examples/metadata/ta_columns.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>column</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t>aar</t>
+  </si>
+  <si>
+    <t>target</t>
+  </si>
+  <si>
+    <t>maal</t>
   </si>
 </sst>
 </file>
@@ -448,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.44140625" customWidth="1"/>
@@ -543,6 +549,14 @@
         <v>20</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update example metadata files
</commit_message>
<xml_diff>
--- a/data/examples/metadata/ta_columns.xlsx
+++ b/data/examples/metadata/ta_columns.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9195"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>column</t>
   </si>
@@ -85,12 +85,6 @@
   </si>
   <si>
     <t>aar</t>
-  </si>
-  <si>
-    <t>target</t>
-  </si>
-  <si>
-    <t>maal</t>
   </si>
 </sst>
 </file>
@@ -454,14 +448,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" customWidth="1"/>
-    <col min="2" max="2" width="33.77734375" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -469,7 +463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -477,7 +471,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -485,7 +479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -493,7 +487,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -501,7 +495,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -509,52 +503,44 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B11" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>